<commit_message>
doc & spreadsheets updated
</commit_message>
<xml_diff>
--- a/testing/AvantisChannelListTesting.xlsx
+++ b/testing/AvantisChannelListTesting.xlsx
@@ -2039,17 +2039,16 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="37" style="2" width="4.29"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="60" min="53" style="2" width="4.29"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="61" min="61" style="3" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="62" style="2" width="4.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="70" min="70" style="3" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="86" min="71" style="2" width="4.29"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="94" min="87" style="2" width="4.29"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="69" min="62" style="2" width="4.29"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="70" min="70" style="3" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="94" min="71" style="2" width="4.29"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="95" min="95" style="2" width="11"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="103" min="96" style="2" width="4.29"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="107" min="104" style="2" width="3.56"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="108" min="108" style="2" width="10.42"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="116" min="109" style="2" width="4.29"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="120" min="117" style="2" width="3.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="121" min="121" style="2" width="12.01"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="121" min="121" style="2" width="12.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="122" min="122" style="3" width="35.84"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="136" min="123" style="2" width="11"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="145" min="138" style="2" width="10.98"/>

</xml_diff>